<commit_message>
Fix verified audit issues, enhance raster statistics, and support dual-runtime master Excel guide
</commit_message>
<xml_diff>
--- a/Fields_AR_EN_Units.xlsx
+++ b/Fields_AR_EN_Units.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1068,3605 +1068,3640 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="10" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Measurement_Unit</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Admin / إدارة البيانات</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>وحدة القياس المعتمدة للمتغير (Measurement Unit).</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>نص</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>T_AnnMean</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>T_Annual_Mean</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>المتوسط الحسابي السنوي لدرجة حرارة الهواء عند ارتفاع 2 متر لجميع شهور السنة.</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لدرجة الحرارة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="17" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>T_WinMean</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>T_Winter_Mean</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة الهواء لفصل الشتاء الأرصادي (شهور ديسمبر، يناير، فبراير - DJF).</t>
         </is>
       </c>
-      <c r="F15" s="22" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G15" s="23" t="inlineStr">
+      <c r="G16" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة الحرارة خلال فصل الشتاء (°C)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>T_SprMean</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>T_Spring_Mean</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة الهواء لفصل الربيع الأرصادي (شهور مارس، أبريل، مايو - MAM).</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة الحرارة خلال فصل الربيع (°C)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>T_SumMean</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>T_Summer_Mean</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة الهواء لفصل الصيف الأرصادي (شهور يونيو، يوليو، أغسطس - JJA).</t>
         </is>
       </c>
-      <c r="F17" s="22" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G17" s="23" t="inlineStr">
+      <c r="G18" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة الحرارة خلال فصل الصيف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>T_AutMean</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>T_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة الهواء لفصل الخريف الأرصادي (شهور سبتمبر، أكتوبر، نوفمبر - SON).</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة الحرارة خلال فصل الخريف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>T_AnnRng</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>T_Annual_Range</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>المدى الحراري السنوي (الفارق بين متوسط أدفأ شهور السنة ومتوسط أبرد شهور السنة).</t>
         </is>
       </c>
-      <c r="F19" s="22" t="inlineStr">
+      <c r="F20" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G19" s="23" t="inlineStr">
+      <c r="G20" s="23" t="inlineStr">
         <is>
           <t>خريطة المدى الحراري السنوي لدرجات الحرارة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>T_MaxSumMo</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>T_Max_Summer_Month_Mean</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة الحرارة لأدفأ شهور فصل الصيف (أعلى متوسط شهري مسجل في الصيف).</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط أدفأ شهور فصل الصيف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>T_MinWinMo</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>T_Min_Winter_Month_Mean</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة الحرارة لأبرد شهور فصل الشتاء (أدنى متوسط شهري مسجل في الشتاء).</t>
         </is>
       </c>
-      <c r="F21" s="22" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G21" s="23" t="inlineStr">
+      <c r="G22" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط أبرد شهور فصل الشتاء (°C)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>T_MaxMean</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>T_Annual_Max_Mean</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>المتوسط السنوي للنهايات العظمى اليومية لدرجة حرارة الهواء (T2M_MAX).</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي للنهايات العظمى لدرجة الحرارة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>T_MinMean</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>T_Annual_Min_Mean</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>01_Temperature (درجة الحرارة)</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>المتوسط السنوي للنهايات الصغرى اليومية لدرجة حرارة الهواء (T2M_MIN).</t>
         </is>
       </c>
-      <c r="F23" s="22" t="inlineStr">
+      <c r="F24" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G23" s="23" t="inlineStr">
+      <c r="G24" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي للنهايات الصغرى لدرجة الحرارة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>HI_AnnMean</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>HI_Annual_Mean</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>11_Heat_Index (مؤشر الحرارة)</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>المتوسط السنوي لمؤشر الحرارة المحسوسة المحسوب بمعادلة روتفوش وستيدمان للحرارة والرطوبة.</t>
         </is>
       </c>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G24" s="16" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لمؤشر الحرارة المحسوسة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>HI_SumMean</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C26" s="19" t="inlineStr">
         <is>
           <t>HI_Summer_Mean</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>11_Heat_Index (مؤشر الحرارة)</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>متوسط مؤشر الحرارة المحسوسة خلال فصل الصيف (مقياس الإجهاد الحراري الفعلي).</t>
         </is>
       </c>
-      <c r="F25" s="22" t="inlineStr">
+      <c r="F26" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G25" s="23" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الحرارة المحسوسة خلال فصل الصيف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>HI_WinMean</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>HI_Winter_Mean</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>11_Heat_Index (مؤشر الحرارة)</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>متوسط مؤشر الحرارة الظاهرية/الهيوميدكس خلال فصل الشتاء في الأجواء الباردة والرطبة.</t>
         </is>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G26" s="16" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة الحرارة المحسوسة خلال فصل الشتاء (°C)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>HI_AnRng</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C28" s="19" t="inlineStr">
         <is>
           <t>HI_Annual_Range</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>11_Heat_Index (مؤشر الحرارة)</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>المدى السنوي لمؤشر الحرارة المحسوسة (الفارق بين أعلى شهر إجهاد حراري وأدنى شهر).</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G27" s="23" t="inlineStr">
+      <c r="G28" s="23" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لمؤشر الحرارة المحسوسة (°C)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>WBGT_SuMn</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>WBGT_Summer_Mean</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>11_Heat_Index (مؤشر الحرارة)</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة البصيلة الرطبة الكروية الصيفي في الظل (معيار ISO 7243 للإجهاد المهني والرياضي).</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G28" s="16" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الإجهاد الحراري الصيفي (WBGT) (°C)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>Td_AnnMean</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>Td_Annual_Mean</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>المتوسط الحسابي السنوي لدرجة حرارة نقطة الندى عند ارتفاع 2 متر.</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G29" s="23" t="inlineStr">
+      <c r="G30" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لدرجة حرارة نقطة الندى (°C)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Td_WinMean</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Td_Winter_Mean</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة نقطة الندى خلال فصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G30" s="16" t="inlineStr">
+      <c r="G31" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة حرارة نقطة الندى خلال فصل الشتاء (°C)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>Td_SprMean</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>Td_Spring_Mean</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة نقطة الندى خلال فصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G31" s="23" t="inlineStr">
+      <c r="G32" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة حرارة نقطة الندى خلال فصل الربيع (°C)</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Td_SumMean</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>Td_Summer_Mean</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة نقطة الندى خلال فصل الصيف الأرصادي (JJA - مؤشر مباشر للرطوبة الخانقة والكتمة).</t>
         </is>
       </c>
-      <c r="F32" s="15" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="G33" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة حرارة نقطة الندى خلال فصل الصيف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="17" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="18" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>Td_AutMean</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C34" s="19" t="inlineStr">
         <is>
           <t>Td_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة حرارة نقطة الندى خلال فصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F33" s="22" t="inlineStr">
+      <c r="F34" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G33" s="23" t="inlineStr">
+      <c r="G34" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط درجة حرارة نقطة الندى خلال فصل الخريف (°C)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Td_AnnRng</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>Td_Annual_Range</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>07_Dew_Point (نقطة الندى)</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي لدرجة حرارة نقطة الندى (الفارق بين أعلى وأدنى متوسط شهري لنقطة الندى).</t>
         </is>
       </c>
-      <c r="F34" s="15" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G34" s="16" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لدرجة حرارة نقطة الندى (°C)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="17" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>R_AnnTot</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C36" s="19" t="inlineStr">
         <is>
           <t>R_Annual_Total</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>المجموع التراكمي السنوي لتساقط الأمطار (مجموع كميات الهطول لجميع شهور السنة).</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F36" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G35" s="23" t="inlineStr">
+      <c r="G36" s="23" t="inlineStr">
         <is>
           <t>خريطة المجموع السنوي لتساقط الأمطار (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>R_AnnMean</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>R_Annual_Mean</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>المعدل الشهري لتساقط الأمطار (المجموع التراكمي السنوي مقسوماً على 12 شهراً).</t>
         </is>
       </c>
-      <c r="F36" s="15" t="inlineStr">
+      <c r="F37" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G36" s="16" t="inlineStr">
+      <c r="G37" s="16" t="inlineStr">
         <is>
           <t>خريطة المعدل الشهري لتساقط الأمطار (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="17" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="18" t="inlineStr">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>R_AnnRng</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C38" s="19" t="inlineStr">
         <is>
           <t>R_Annual_Range</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>المدى السنوي لتساقط الأمطار (الفارق بين أعلى شهر مطراً وأقل شهر مطراً في السنة).</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F38" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G37" s="23" t="inlineStr">
+      <c r="G38" s="23" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لتساقط الأمطار (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="10" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>R_SeaRng</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>R_Seasonal_Range</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr">
         <is>
           <t>المدى الفصلي لتساقط الأمطار (الفارق بين مجموع أعلى فصول السنة مطراً ومجموع أقلها مطراً).</t>
         </is>
       </c>
-      <c r="F38" s="15" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G38" s="16" t="inlineStr">
+      <c r="G39" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى الفصلي لتساقط الأمطار (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="17" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="18" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="18" t="inlineStr">
         <is>
           <t>R_WinTot</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="C40" s="19" t="inlineStr">
         <is>
           <t>R_Winter_Total</t>
         </is>
       </c>
-      <c r="D39" s="20" t="inlineStr">
+      <c r="D40" s="20" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>المجموع التراكمي لأمطار فصل الشتاء الأرصادي (شهور ديسمبر، يناير، فبراير - DJF).</t>
         </is>
       </c>
-      <c r="F39" s="22" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G39" s="23" t="inlineStr">
+      <c r="G40" s="23" t="inlineStr">
         <is>
           <t>خريطة مجموع تساقط الأمطار خلال فصل الشتاء (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>R_SprTot</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>R_Spring_Total</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t>المجموع التراكمي لأمطار فصل الربيع الأرصادي (شهور مارس، أبريل، مايو - MAM).</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G40" s="16" t="inlineStr">
+      <c r="G41" s="16" t="inlineStr">
         <is>
           <t>خريطة مجموع تساقط الأمطار خلال فصل الربيع (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="24" customHeight="1">
-      <c r="A41" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="18" t="inlineStr">
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="17" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>R_SumTot</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C42" s="19" t="inlineStr">
         <is>
           <t>R_Summer_Total</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E41" s="21" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>المجموع التراكمي لأمطار فصل الصيف الأرصادي (شهور يونيو، يوليو، أغسطس - JJA).</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G41" s="23" t="inlineStr">
+      <c r="G42" s="23" t="inlineStr">
         <is>
           <t>خريطة مجموع تساقط الأمطار خلال فصل الصيف (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>R_AutTot</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>R_Autumn_Total</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>02_Precipitation (الأمطار)</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>المجموع التراكمي لأمطار فصل الخريف الأرصادي (شهور سبتمبر، أكتوبر، نوفمبر - SON).</t>
         </is>
       </c>
-      <c r="F42" s="15" t="inlineStr">
+      <c r="F43" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G42" s="16" t="inlineStr">
+      <c r="G43" s="16" t="inlineStr">
         <is>
           <t>خريطة مجموع تساقط الأمطار خلال فصل الخريف (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="17" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="18" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
         <is>
           <t>PSL_AnMean</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C44" s="19" t="inlineStr">
         <is>
           <t>PSL_Annual_Mean</t>
         </is>
       </c>
-      <c r="D43" s="20" t="inlineStr">
+      <c r="D44" s="20" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E43" s="21" t="inlineStr">
+      <c r="E44" s="21" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي السنوي المصحح عند مستوى سطح البحر القياسي (Sea Level Pressure).</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G43" s="23" t="inlineStr">
+      <c r="G44" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الضغط الجوي عند مستوى سطح البحر (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>PSL_WnMean</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>PSL_Winter_Mean</t>
         </is>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي عند مستوى سطح البحر لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F44" s="15" t="inlineStr">
+      <c r="F45" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G44" s="16" t="inlineStr">
+      <c r="G45" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط ضغط مستوى سطح البحر خلال فصل الشتاء (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="17" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t>PSL_SpMean</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C46" s="19" t="inlineStr">
         <is>
           <t>PSL_Spring_Mean</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E45" s="21" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي عند مستوى سطح البحر لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G45" s="23" t="inlineStr">
+      <c r="G46" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط ضغط مستوى سطح البحر خلال فصل الربيع (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>PSL_SuMean</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>PSL_Summer_Mean</t>
         </is>
       </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي عند مستوى سطح البحر لفصل الصيف الأرصادي (JJA).</t>
         </is>
       </c>
-      <c r="F46" s="15" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G46" s="16" t="inlineStr">
+      <c r="G47" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط ضغط مستوى سطح البحر خلال فصل الصيف (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="24" customHeight="1">
-      <c r="A47" s="17" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="17" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
         <is>
           <t>PSL_AuMean</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C48" s="19" t="inlineStr">
         <is>
           <t>PSL_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D47" s="20" t="inlineStr">
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي عند مستوى سطح البحر لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G47" s="23" t="inlineStr">
+      <c r="G48" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط ضغط مستوى سطح البحر خلال فصل الخريف (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="11" t="inlineStr">
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>PSL_AnRng</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>PSL_Annual_Range</t>
         </is>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D49" s="13" t="inlineStr">
         <is>
           <t>03_Sea_Level_Pressure (ضغط مستوى البحر)</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="E49" s="14" t="inlineStr">
         <is>
           <t>المدى البارومتري السنوي لضغط مستوى البحر (الفارق بين أعلى وأدنى متوسط شهري للضغط).</t>
         </is>
       </c>
-      <c r="F48" s="15" t="inlineStr">
+      <c r="F49" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G48" s="16" t="inlineStr">
+      <c r="G49" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لضغط مستوى سطح البحر (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="17" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
         <is>
           <t>PS_AnnMean</t>
         </is>
       </c>
-      <c r="C49" s="19" t="inlineStr">
+      <c r="C50" s="19" t="inlineStr">
         <is>
           <t>PS_Annual_Mean</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D50" s="20" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
+      <c r="E50" s="21" t="inlineStr">
         <is>
           <t>المتوسط السنوي للضغط الجوي السطحي الفعلي الحقيقي عند منسوب تضاريس المحطة.</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G49" s="23" t="inlineStr">
+      <c r="G50" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي للضغط الجوي السطحي (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="11" t="inlineStr">
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>PS_WinMean</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>PS_Winter_Mean</t>
         </is>
       </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="D51" s="13" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E51" s="14" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي السطحي الفعلي لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F50" s="15" t="inlineStr">
+      <c r="F51" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G50" s="16" t="inlineStr">
+      <c r="G51" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الضغط السطحي خلال فصل الشتاء (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
         <is>
           <t>PS_SprMean</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C52" s="19" t="inlineStr">
         <is>
           <t>PS_Spring_Mean</t>
         </is>
       </c>
-      <c r="D51" s="20" t="inlineStr">
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E51" s="21" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي السطحي الفعلي لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G51" s="23" t="inlineStr">
+      <c r="G52" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الضغط السطحي خلال فصل الربيع (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="24" customHeight="1">
-      <c r="A52" s="10" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="11" t="inlineStr">
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>PS_SumMean</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>PS_Summer_Mean</t>
         </is>
       </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="D53" s="13" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
+      <c r="E53" s="14" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي السطحي الفعلي لفصل الصيف الأرصادي (JJA).</t>
         </is>
       </c>
-      <c r="F52" s="15" t="inlineStr">
+      <c r="F53" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G52" s="16" t="inlineStr">
+      <c r="G53" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الضغط السطحي خلال فصل الصيف (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="17" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="18" t="inlineStr">
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
         <is>
           <t>PS_AutMean</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C54" s="19" t="inlineStr">
         <is>
           <t>PS_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D53" s="20" t="inlineStr">
+      <c r="D54" s="20" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E53" s="21" t="inlineStr">
+      <c r="E54" s="21" t="inlineStr">
         <is>
           <t>متوسط الضغط الجوي السطحي الفعلي لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G53" s="23" t="inlineStr">
+      <c r="G54" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الضغط السطحي خلال فصل الخريف (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="10" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="11" t="inlineStr">
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>PS_AnnRng</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
         <is>
           <t>PS_Annual_Range</t>
         </is>
       </c>
-      <c r="D54" s="13" t="inlineStr">
+      <c r="D55" s="13" t="inlineStr">
         <is>
           <t>04_Surface_Pressure (الضغط السطحي)</t>
         </is>
       </c>
-      <c r="E54" s="14" t="inlineStr">
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>المدى البارومتري السنوي للضغط السطحي (الفارق بين أعلى وأدنى متوسط شهري للضغط السطحي).</t>
         </is>
       </c>
-      <c r="F54" s="15" t="inlineStr">
+      <c r="F55" s="15" t="inlineStr">
         <is>
           <t>hPa / mbar</t>
         </is>
       </c>
-      <c r="G54" s="16" t="inlineStr">
+      <c r="G55" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي للضغط الجوي السطحي (hPa)</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="17" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="18" t="inlineStr">
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="17" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
         <is>
           <t>WSp_AnMean</t>
         </is>
       </c>
-      <c r="C55" s="19" t="inlineStr">
+      <c r="C56" s="19" t="inlineStr">
         <is>
           <t>W_Spd_Annual_Mean</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr">
+      <c r="D56" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E55" s="21" t="inlineStr">
+      <c r="E56" s="21" t="inlineStr">
         <is>
           <t>المتوسط السنوي لسرعة الرياح عند ارتفاع 10 أمتار فوق سطح الأرض.</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G55" s="23" t="inlineStr">
+      <c r="G56" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لسرعة الرياح (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="10" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="11" t="inlineStr">
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
         <is>
           <t>WSp_WnMean</t>
         </is>
       </c>
-      <c r="C56" s="12" t="inlineStr">
+      <c r="C57" s="12" t="inlineStr">
         <is>
           <t>W_Spd_Winter_Mean</t>
         </is>
       </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="D57" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E56" s="14" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>متوسط سرعة الرياح لفصل الشتاء الأرصادي عند ارتفاع 10 أمتار (DJF).</t>
         </is>
       </c>
-      <c r="F56" s="15" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G56" s="16" t="inlineStr">
+      <c r="G57" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط سرعة الرياح خلال فصل الشتاء (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="24" customHeight="1">
-      <c r="A57" s="17" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="17" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
         <is>
           <t>WSp_SpMean</t>
         </is>
       </c>
-      <c r="C57" s="19" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>W_Spd_Spring_Mean</t>
         </is>
       </c>
-      <c r="D57" s="20" t="inlineStr">
+      <c r="D58" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E57" s="21" t="inlineStr">
+      <c r="E58" s="21" t="inlineStr">
         <is>
           <t>متوسط سرعة الرياح لفصل الربيع الأرصادي عند ارتفاع 10 أمتار (MAM).</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G57" s="23" t="inlineStr">
+      <c r="G58" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط سرعة الرياح خلال فصل الربيع (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="10" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="11" t="inlineStr">
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="10" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>WSp_SuMean</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>W_Spd_Summer_Mean</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D59" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E58" s="14" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t>متوسط سرعة الرياح لفصل الصيف الأرصادي عند ارتفاع 10 أمتار (JJA).</t>
         </is>
       </c>
-      <c r="F58" s="15" t="inlineStr">
+      <c r="F59" s="15" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G58" s="16" t="inlineStr">
+      <c r="G59" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط سرعة الرياح خلال فصل الصيف (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="17" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
+    <row r="60" ht="24" customHeight="1">
+      <c r="A60" s="17" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
         <is>
           <t>WSp_AuMean</t>
         </is>
       </c>
-      <c r="C59" s="19" t="inlineStr">
+      <c r="C60" s="19" t="inlineStr">
         <is>
           <t>W_Spd_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D59" s="20" t="inlineStr">
+      <c r="D60" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E59" s="21" t="inlineStr">
+      <c r="E60" s="21" t="inlineStr">
         <is>
           <t>متوسط سرعة الرياح لفصل الخريف الأرصادي عند ارتفاع 10 أمتار (SON).</t>
         </is>
       </c>
-      <c r="F59" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G59" s="23" t="inlineStr">
+      <c r="G60" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط سرعة الرياح خلال فصل الخريف (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="10" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="11" t="inlineStr">
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>WSp_MaxMo</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>W_Spd_Annual_Max_Month</t>
         </is>
       </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="D61" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t>أقصى متوسط شهري مسجل لسرعة الرياح في السنة (ذروة النشاط الريحي).</t>
         </is>
       </c>
-      <c r="F60" s="15" t="inlineStr">
+      <c r="F61" s="15" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G60" s="16" t="inlineStr">
+      <c r="G61" s="16" t="inlineStr">
         <is>
           <t>خريطة أقصى متوسط شهري لسرعة الرياح (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="24" customHeight="1">
-      <c r="A61" s="17" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
+    <row r="62" ht="24" customHeight="1">
+      <c r="A62" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
         <is>
           <t>WSp_MinMo</t>
         </is>
       </c>
-      <c r="C61" s="19" t="inlineStr">
+      <c r="C62" s="19" t="inlineStr">
         <is>
           <t>W_Spd_Annual_Min_Month</t>
         </is>
       </c>
-      <c r="D61" s="20" t="inlineStr">
+      <c r="D62" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E61" s="21" t="inlineStr">
+      <c r="E62" s="21" t="inlineStr">
         <is>
           <t>أدنى متوسط شهري مسجل لسرعة الرياح في السنة (فترة الهدوء الريحي).</t>
         </is>
       </c>
-      <c r="F61" s="22" t="inlineStr">
+      <c r="F62" s="22" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G61" s="23" t="inlineStr">
+      <c r="G62" s="23" t="inlineStr">
         <is>
           <t>خريطة أدنى متوسط شهري لسرعة الرياح (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="24" customHeight="1">
-      <c r="A62" s="10" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="11" t="inlineStr">
+    <row r="63" ht="24" customHeight="1">
+      <c r="A63" s="10" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
         <is>
           <t>WSp_AnRng</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
         <is>
           <t>W_Spd_Annual_Range</t>
         </is>
       </c>
-      <c r="D62" s="13" t="inlineStr">
+      <c r="D63" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="E63" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي لسرعة الرياح (الفارق بين أشد شهور السنة رياحاً وأهدأها سرعة).</t>
         </is>
       </c>
-      <c r="F62" s="15" t="inlineStr">
+      <c r="F63" s="15" t="inlineStr">
         <is>
           <t>م/ث (m/s)</t>
         </is>
       </c>
-      <c r="G62" s="16" t="inlineStr">
+      <c r="G63" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لسرعة الرياح (م/ث)</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="24" customHeight="1">
-      <c r="A63" s="17" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
+    <row r="64" ht="24" customHeight="1">
+      <c r="A64" s="17" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
         <is>
           <t>WDr_AnMean</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
+      <c r="C64" s="19" t="inlineStr">
         <is>
           <t>W_Dir_Annual_Mean</t>
         </is>
       </c>
-      <c r="D63" s="20" t="inlineStr">
+      <c r="D64" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E63" s="21" t="inlineStr">
+      <c r="E64" s="21" t="inlineStr">
         <is>
           <t>الاتجاه السائد السنوي للرياح بالدرجات الزاوية (محسوب بالمتوسط الدائري للمتجهات الدائرية atan2).</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
+      <c r="F64" s="22" t="inlineStr">
         <is>
           <t>درجة (°)</t>
         </is>
       </c>
-      <c r="G63" s="23" t="inlineStr">
+      <c r="G64" s="23" t="inlineStr">
         <is>
           <t>خريطة الاتجاه السائد السنوي للرياح (درجات)</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="24" customHeight="1">
-      <c r="A64" s="10" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
+    <row r="65" ht="24" customHeight="1">
+      <c r="A65" s="10" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>WDr_WnMean</t>
         </is>
       </c>
-      <c r="C64" s="12" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>W_Dir_Winter_Mean</t>
         </is>
       </c>
-      <c r="D64" s="13" t="inlineStr">
+      <c r="D65" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E64" s="14" t="inlineStr">
+      <c r="E65" s="14" t="inlineStr">
         <is>
           <t>اتجاه الرياح السائد خلال فصل الشتاء الأرصادي بالدرجات الزاوية (DJF).</t>
         </is>
       </c>
-      <c r="F64" s="15" t="inlineStr">
+      <c r="F65" s="15" t="inlineStr">
         <is>
           <t>درجة (°)</t>
         </is>
       </c>
-      <c r="G64" s="16" t="inlineStr">
+      <c r="G65" s="16" t="inlineStr">
         <is>
           <t>خريطة اتجاه الرياح السائد خلال فصل الشتاء (درجات)</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="24" customHeight="1">
-      <c r="A65" s="17" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="18" t="inlineStr">
+    <row r="66" ht="24" customHeight="1">
+      <c r="A66" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
         <is>
           <t>WDr_SpMean</t>
         </is>
       </c>
-      <c r="C65" s="19" t="inlineStr">
+      <c r="C66" s="19" t="inlineStr">
         <is>
           <t>W_Dir_Spring_Mean</t>
         </is>
       </c>
-      <c r="D65" s="20" t="inlineStr">
+      <c r="D66" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E65" s="21" t="inlineStr">
+      <c r="E66" s="21" t="inlineStr">
         <is>
           <t>اتجاه الرياح السائد خلال فصل الربيع الأرصادي بالدرجات الزاوية (MAM).</t>
         </is>
       </c>
-      <c r="F65" s="22" t="inlineStr">
+      <c r="F66" s="22" t="inlineStr">
         <is>
           <t>درجة (°)</t>
         </is>
       </c>
-      <c r="G65" s="23" t="inlineStr">
+      <c r="G66" s="23" t="inlineStr">
         <is>
           <t>خريطة اتجاه الرياح السائد خلال فصل الربيع (درجات)</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="24" customHeight="1">
-      <c r="A66" s="10" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="11" t="inlineStr">
+    <row r="67" ht="24" customHeight="1">
+      <c r="A67" s="10" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>WDr_SuMean</t>
         </is>
       </c>
-      <c r="C66" s="12" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>W_Dir_Summer_Mean</t>
         </is>
       </c>
-      <c r="D66" s="13" t="inlineStr">
+      <c r="D67" s="13" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E66" s="14" t="inlineStr">
+      <c r="E67" s="14" t="inlineStr">
         <is>
           <t>اتجاه الرياح السائد خلال فصل الصيف الأرصادي بالدرجات الزاوية (JJA).</t>
         </is>
       </c>
-      <c r="F66" s="15" t="inlineStr">
+      <c r="F67" s="15" t="inlineStr">
         <is>
           <t>درجة (°)</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
+      <c r="G67" s="16" t="inlineStr">
         <is>
           <t>خريطة اتجاه الرياح السائد خلال فصل الصيف (درجات)</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="24" customHeight="1">
-      <c r="A67" s="17" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="18" t="inlineStr">
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
         <is>
           <t>WDr_AuMean</t>
         </is>
       </c>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>W_Dir_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D67" s="20" t="inlineStr">
+      <c r="D68" s="20" t="inlineStr">
         <is>
           <t>05_Wind (الرياح)</t>
         </is>
       </c>
-      <c r="E67" s="21" t="inlineStr">
+      <c r="E68" s="21" t="inlineStr">
         <is>
           <t>اتجاه الرياح السائد خلال فصل الخريف الأرصادي بالدرجات الزاوية (SON).</t>
         </is>
       </c>
-      <c r="F67" s="22" t="inlineStr">
+      <c r="F68" s="22" t="inlineStr">
         <is>
           <t>درجة (°)</t>
         </is>
       </c>
-      <c r="G67" s="23" t="inlineStr">
+      <c r="G68" s="23" t="inlineStr">
         <is>
           <t>خريطة اتجاه الرياح السائد خلال فصل الخريف (درجات)</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="24" customHeight="1">
-      <c r="A68" s="10" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="10" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>RH_AnMean</t>
         </is>
       </c>
-      <c r="C68" s="12" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
         <is>
           <t>RH_Annual_Mean</t>
         </is>
       </c>
-      <c r="D68" s="13" t="inlineStr">
+      <c r="D69" s="13" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E68" s="14" t="inlineStr">
+      <c r="E69" s="14" t="inlineStr">
         <is>
           <t>المتوسط الحسابي السنوي للرطوبة النسبية للهواء عند ارتفاع 2 متر كنسبة مئوية.</t>
         </is>
       </c>
-      <c r="F68" s="15" t="inlineStr">
+      <c r="F69" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G68" s="16" t="inlineStr">
+      <c r="G69" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي للرطوبة النسبية (%)</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="24" customHeight="1">
-      <c r="A69" s="17" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="18" t="inlineStr">
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="17" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
         <is>
           <t>RH_WnMean</t>
         </is>
       </c>
-      <c r="C69" s="19" t="inlineStr">
+      <c r="C70" s="19" t="inlineStr">
         <is>
           <t>RH_Winter_Mean</t>
         </is>
       </c>
-      <c r="D69" s="20" t="inlineStr">
+      <c r="D70" s="20" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E69" s="21" t="inlineStr">
+      <c r="E70" s="21" t="inlineStr">
         <is>
           <t>متوسط الرطوبة النسبية لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F69" s="22" t="inlineStr">
+      <c r="F70" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G69" s="23" t="inlineStr">
+      <c r="G70" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الرطوبة النسبية خلال فصل الشتاء (%)</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="24" customHeight="1">
-      <c r="A70" s="10" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="11" t="inlineStr">
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
         <is>
           <t>RH_SpMean</t>
         </is>
       </c>
-      <c r="C70" s="12" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
         <is>
           <t>RH_Spring_Mean</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D71" s="13" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E70" s="14" t="inlineStr">
+      <c r="E71" s="14" t="inlineStr">
         <is>
           <t>متوسط الرطوبة النسبية لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F70" s="15" t="inlineStr">
+      <c r="F71" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G70" s="16" t="inlineStr">
+      <c r="G71" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الرطوبة النسبية خلال فصل الربيع (%)</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="24" customHeight="1">
-      <c r="A71" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="18" t="inlineStr">
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="17" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
         <is>
           <t>RH_SuMean</t>
         </is>
       </c>
-      <c r="C71" s="19" t="inlineStr">
+      <c r="C72" s="19" t="inlineStr">
         <is>
           <t>RH_Summer_Mean</t>
         </is>
       </c>
-      <c r="D71" s="20" t="inlineStr">
+      <c r="D72" s="20" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E71" s="21" t="inlineStr">
+      <c r="E72" s="21" t="inlineStr">
         <is>
           <t>متوسط الرطوبة النسبية لفصل الصيف الأرصادي (JJA).</t>
         </is>
       </c>
-      <c r="F71" s="22" t="inlineStr">
+      <c r="F72" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G71" s="23" t="inlineStr">
+      <c r="G72" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الرطوبة النسبية خلال فصل الصيف (%)</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="24" customHeight="1">
-      <c r="A72" s="10" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" s="11" t="inlineStr">
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
         <is>
           <t>RH_AuMean</t>
         </is>
       </c>
-      <c r="C72" s="12" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
         <is>
           <t>RH_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D72" s="13" t="inlineStr">
+      <c r="D73" s="13" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E72" s="14" t="inlineStr">
+      <c r="E73" s="14" t="inlineStr">
         <is>
           <t>متوسط الرطوبة النسبية لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F72" s="15" t="inlineStr">
+      <c r="F73" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
+      <c r="G73" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الرطوبة النسبية خلال فصل الخريف (%)</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="24" customHeight="1">
-      <c r="A73" s="17" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" s="18" t="inlineStr">
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
         <is>
           <t>RH_AnRng</t>
         </is>
       </c>
-      <c r="C73" s="19" t="inlineStr">
+      <c r="C74" s="19" t="inlineStr">
         <is>
           <t>RH_Annual_Range</t>
         </is>
       </c>
-      <c r="D73" s="20" t="inlineStr">
+      <c r="D74" s="20" t="inlineStr">
         <is>
           <t>06_Relative_Humidity (الرطوبة النسبية)</t>
         </is>
       </c>
-      <c r="E73" s="21" t="inlineStr">
+      <c r="E74" s="21" t="inlineStr">
         <is>
           <t>المدى السنوي للرطوبة النسبية (الفارق بين أعلى شهر رطوبة وأدنى شهر رطوبة).</t>
         </is>
       </c>
-      <c r="F73" s="22" t="inlineStr">
+      <c r="F74" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G73" s="23" t="inlineStr">
+      <c r="G74" s="23" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي للرطوبة النسبية (%)</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="24" customHeight="1">
-      <c r="A74" s="10" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="11" t="inlineStr">
+    <row r="75" ht="24" customHeight="1">
+      <c r="A75" s="10" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
         <is>
           <t>Sol_AnMean</t>
         </is>
       </c>
-      <c r="C74" s="12" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
         <is>
           <t>Sol_Annual_Mean</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D75" s="13" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E74" s="14" t="inlineStr">
+      <c r="E75" s="14" t="inlineStr">
         <is>
           <t>المتوسط اليومي السنوي للإشعاع الشمسي الكلي السطحي الواصل لسطح الأرض في كافة ظروف السماء.</t>
         </is>
       </c>
-      <c r="F74" s="15" t="inlineStr">
+      <c r="F75" s="15" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G74" s="16" t="inlineStr">
+      <c r="G75" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط اليومي السنوي للإشعاع الشمسي (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="24" customHeight="1">
-      <c r="A75" s="17" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="18" t="inlineStr">
+    <row r="76" ht="24" customHeight="1">
+      <c r="A76" s="17" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
         <is>
           <t>Sol_AnTot</t>
         </is>
       </c>
-      <c r="C75" s="19" t="inlineStr">
+      <c r="C76" s="19" t="inlineStr">
         <is>
           <t>Sol_Annual_Total</t>
         </is>
       </c>
-      <c r="D75" s="20" t="inlineStr">
+      <c r="D76" s="20" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E75" s="21" t="inlineStr">
+      <c r="E76" s="21" t="inlineStr">
         <is>
           <t>إجمالي الطاقة الشمسية السنوية التراكمية الساقطة على المتر المربع في السنة كاملة.</t>
         </is>
       </c>
-      <c r="F75" s="22" t="inlineStr">
+      <c r="F76" s="22" t="inlineStr">
         <is>
           <t>kWh/m²/year</t>
         </is>
       </c>
-      <c r="G75" s="23" t="inlineStr">
+      <c r="G76" s="23" t="inlineStr">
         <is>
           <t>خريطة إجمالي الطاقة الشمسية السنوية التراكمية (kWh/m²/year)</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="24" customHeight="1">
-      <c r="A76" s="10" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="11" t="inlineStr">
+    <row r="77" ht="24" customHeight="1">
+      <c r="A77" s="10" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>Sol_WnMean</t>
         </is>
       </c>
-      <c r="C76" s="12" t="inlineStr">
+      <c r="C77" s="12" t="inlineStr">
         <is>
           <t>Sol_Winter_Mean</t>
         </is>
       </c>
-      <c r="D76" s="13" t="inlineStr">
+      <c r="D77" s="13" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E76" s="14" t="inlineStr">
+      <c r="E77" s="14" t="inlineStr">
         <is>
           <t>متوسط الإشعاع الشمسي اليومي لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F76" s="15" t="inlineStr">
+      <c r="F77" s="15" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G76" s="16" t="inlineStr">
+      <c r="G77" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الإشعاع الشمسي خلال فصل الشتاء (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="24" customHeight="1">
-      <c r="A77" s="17" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" s="18" t="inlineStr">
+    <row r="78" ht="24" customHeight="1">
+      <c r="A78" s="17" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
         <is>
           <t>Sol_SpMean</t>
         </is>
       </c>
-      <c r="C77" s="19" t="inlineStr">
+      <c r="C78" s="19" t="inlineStr">
         <is>
           <t>Sol_Spring_Mean</t>
         </is>
       </c>
-      <c r="D77" s="20" t="inlineStr">
+      <c r="D78" s="20" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E77" s="21" t="inlineStr">
+      <c r="E78" s="21" t="inlineStr">
         <is>
           <t>متوسط الإشعاع الشمسي اليومي لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F77" s="22" t="inlineStr">
+      <c r="F78" s="22" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G77" s="23" t="inlineStr">
+      <c r="G78" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الإشعاع الشمسي خلال فصل الربيع (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="24" customHeight="1">
-      <c r="A78" s="10" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" s="11" t="inlineStr">
+    <row r="79" ht="24" customHeight="1">
+      <c r="A79" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
         <is>
           <t>Sol_SuMean</t>
         </is>
       </c>
-      <c r="C78" s="12" t="inlineStr">
+      <c r="C79" s="12" t="inlineStr">
         <is>
           <t>Sol_Summer_Mean</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D79" s="13" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E78" s="14" t="inlineStr">
+      <c r="E79" s="14" t="inlineStr">
         <is>
           <t>متوسط الإشعاع الشمسي اليومي لفصل الصيف الأرصادي (JJA).</t>
         </is>
       </c>
-      <c r="F78" s="15" t="inlineStr">
+      <c r="F79" s="15" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G78" s="16" t="inlineStr">
+      <c r="G79" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الإشعاع الشمسي خلال فصل الصيف (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="24" customHeight="1">
-      <c r="A79" s="17" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" s="18" t="inlineStr">
+    <row r="80" ht="24" customHeight="1">
+      <c r="A80" s="17" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
         <is>
           <t>Sol_AuMean</t>
         </is>
       </c>
-      <c r="C79" s="19" t="inlineStr">
+      <c r="C80" s="19" t="inlineStr">
         <is>
           <t>Sol_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D79" s="20" t="inlineStr">
+      <c r="D80" s="20" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E79" s="21" t="inlineStr">
+      <c r="E80" s="21" t="inlineStr">
         <is>
           <t>متوسط الإشعاع الشمسي اليومي لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F79" s="22" t="inlineStr">
+      <c r="F80" s="22" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G79" s="23" t="inlineStr">
+      <c r="G80" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الإشعاع الشمسي خلال فصل الخريف (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="24" customHeight="1">
-      <c r="A80" s="10" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="11" t="inlineStr">
+    <row r="81" ht="24" customHeight="1">
+      <c r="A81" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
         <is>
           <t>Sol_AnRng</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr">
+      <c r="C81" s="12" t="inlineStr">
         <is>
           <t>Sol_Annual_Range</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D81" s="13" t="inlineStr">
         <is>
           <t>08_Solar_Radiation (الإشعاع الشمسي)</t>
         </is>
       </c>
-      <c r="E80" s="14" t="inlineStr">
+      <c r="E81" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي للإشعاع الشمسي (الفارق بين ذروة الإشعاع في الصيف وأدناه في الشتاء).</t>
         </is>
       </c>
-      <c r="F80" s="15" t="inlineStr">
+      <c r="F81" s="15" t="inlineStr">
         <is>
           <t>kWh/m²/day</t>
         </is>
       </c>
-      <c r="G80" s="16" t="inlineStr">
+      <c r="G81" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي للإشعاع الشمسي (kWh/m²/day)</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="24" customHeight="1">
-      <c r="A81" s="17" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" s="18" t="inlineStr">
+    <row r="82" ht="24" customHeight="1">
+      <c r="A82" s="17" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
         <is>
           <t>UV_AnMean</t>
         </is>
       </c>
-      <c r="C81" s="19" t="inlineStr">
+      <c r="C82" s="19" t="inlineStr">
         <is>
           <t>UV_Annual_Mean</t>
         </is>
       </c>
-      <c r="D81" s="20" t="inlineStr">
+      <c r="D82" s="20" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E81" s="21" t="inlineStr">
+      <c r="E82" s="21" t="inlineStr">
         <is>
           <t>المتوسط السنوي لمؤشر الأشعة فوق البنفسجية عند الظهيرة وفق منظومة منظمة الصحة العالمية.</t>
         </is>
       </c>
-      <c r="F81" s="22" t="inlineStr">
+      <c r="F82" s="22" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G81" s="23" t="inlineStr">
+      <c r="G82" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لمؤشر الأشعة فوق البنفسجية (UV)</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="24" customHeight="1">
-      <c r="A82" s="10" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="11" t="inlineStr">
+    <row r="83" ht="24" customHeight="1">
+      <c r="A83" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
         <is>
           <t>UV_WnMean</t>
         </is>
       </c>
-      <c r="C82" s="12" t="inlineStr">
+      <c r="C83" s="12" t="inlineStr">
         <is>
           <t>UV_Winter_Mean</t>
         </is>
       </c>
-      <c r="D82" s="13" t="inlineStr">
+      <c r="D83" s="13" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E82" s="14" t="inlineStr">
+      <c r="E83" s="14" t="inlineStr">
         <is>
           <t>متوسط مؤشر الأشعة فوق البنفسجية لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="F83" s="15" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G82" s="16" t="inlineStr">
+      <c r="G83" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الأشعة فوق البنفسجية خلال فصل الشتاء</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="24" customHeight="1">
-      <c r="A83" s="17" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="18" t="inlineStr">
+    <row r="84" ht="24" customHeight="1">
+      <c r="A84" s="17" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
         <is>
           <t>UV_SpMean</t>
         </is>
       </c>
-      <c r="C83" s="19" t="inlineStr">
+      <c r="C84" s="19" t="inlineStr">
         <is>
           <t>UV_Spring_Mean</t>
         </is>
       </c>
-      <c r="D83" s="20" t="inlineStr">
+      <c r="D84" s="20" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E83" s="21" t="inlineStr">
+      <c r="E84" s="21" t="inlineStr">
         <is>
           <t>متوسط مؤشر الأشعة فوق البنفسجية لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F83" s="22" t="inlineStr">
+      <c r="F84" s="22" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G83" s="23" t="inlineStr">
+      <c r="G84" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الأشعة فوق البنفسجية خلال فصل الربيع</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="24" customHeight="1">
-      <c r="A84" s="10" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="11" t="inlineStr">
+    <row r="85" ht="24" customHeight="1">
+      <c r="A85" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
         <is>
           <t>UV_SuMean</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr">
+      <c r="C85" s="12" t="inlineStr">
         <is>
           <t>UV_Summer_Mean</t>
         </is>
       </c>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="D85" s="13" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E84" s="14" t="inlineStr">
+      <c r="E85" s="14" t="inlineStr">
         <is>
           <t>متوسط مؤشر الأشعة فوق البنفسجية لفصل الصيف الأرصادي (JJA - ذروة مخاطر الحروق الشمسية).</t>
         </is>
       </c>
-      <c r="F84" s="15" t="inlineStr">
+      <c r="F85" s="15" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G84" s="16" t="inlineStr">
+      <c r="G85" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الأشعة فوق البنفسجية خلال فصل الصيف</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="24" customHeight="1">
-      <c r="A85" s="17" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" s="18" t="inlineStr">
+    <row r="86" ht="24" customHeight="1">
+      <c r="A86" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
         <is>
           <t>UV_AuMean</t>
         </is>
       </c>
-      <c r="C85" s="19" t="inlineStr">
+      <c r="C86" s="19" t="inlineStr">
         <is>
           <t>UV_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D85" s="20" t="inlineStr">
+      <c r="D86" s="20" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E85" s="21" t="inlineStr">
+      <c r="E86" s="21" t="inlineStr">
         <is>
           <t>متوسط مؤشر الأشعة فوق البنفسجية لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F85" s="22" t="inlineStr">
+      <c r="F86" s="22" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G85" s="23" t="inlineStr">
+      <c r="G86" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط مؤشر الأشعة فوق البنفسجية خلال فصل الخريف</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="24" customHeight="1">
-      <c r="A86" s="10" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" s="11" t="inlineStr">
+    <row r="87" ht="24" customHeight="1">
+      <c r="A87" s="10" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
         <is>
           <t>UV_AnRng</t>
         </is>
       </c>
-      <c r="C86" s="12" t="inlineStr">
+      <c r="C87" s="12" t="inlineStr">
         <is>
           <t>UV_Annual_Range</t>
         </is>
       </c>
-      <c r="D86" s="13" t="inlineStr">
+      <c r="D87" s="13" t="inlineStr">
         <is>
           <t>09_UV_Index (الأشعة فوق البنفسجية)</t>
         </is>
       </c>
-      <c r="E86" s="14" t="inlineStr">
+      <c r="E87" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي لمؤشر الأشعة فوق البنفسجية (الفارق بين ذروة الصيف وأدنى مستويات الشتاء).</t>
         </is>
       </c>
-      <c r="F86" s="15" t="inlineStr">
+      <c r="F87" s="15" t="inlineStr">
         <is>
           <t>مؤشر (0-16+)</t>
         </is>
       </c>
-      <c r="G86" s="16" t="inlineStr">
+      <c r="G87" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لمؤشر الأشعة فوق البنفسجية</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="17" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="18" t="inlineStr">
+    <row r="88" ht="24" customHeight="1">
+      <c r="A88" s="17" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
         <is>
           <t>Cld_AnMean</t>
         </is>
       </c>
-      <c r="C87" s="19" t="inlineStr">
+      <c r="C88" s="19" t="inlineStr">
         <is>
           <t>Cld_Annual_Mean</t>
         </is>
       </c>
-      <c r="D87" s="20" t="inlineStr">
+      <c r="D88" s="20" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E87" s="21" t="inlineStr">
+      <c r="E88" s="21" t="inlineStr">
         <is>
           <t>المتوسط السنوي لنسبة تغطية السماء بالغيوم والسحب كنسبة مئوية.</t>
         </is>
       </c>
-      <c r="F87" s="22" t="inlineStr">
+      <c r="F88" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G87" s="23" t="inlineStr">
+      <c r="G88" s="23" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لنسبة الغطاء السحابي (%)</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="24" customHeight="1">
-      <c r="A88" s="10" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="11" t="inlineStr">
+    <row r="89" ht="24" customHeight="1">
+      <c r="A89" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
         <is>
           <t>Cld_WnMean</t>
         </is>
       </c>
-      <c r="C88" s="12" t="inlineStr">
+      <c r="C89" s="12" t="inlineStr">
         <is>
           <t>Cld_Winter_Mean</t>
         </is>
       </c>
-      <c r="D88" s="13" t="inlineStr">
+      <c r="D89" s="13" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E88" s="14" t="inlineStr">
+      <c r="E89" s="14" t="inlineStr">
         <is>
           <t>متوسط نسبة تغطية السحب لفصل الشتاء الأرصادي (DJF).</t>
         </is>
       </c>
-      <c r="F88" s="15" t="inlineStr">
+      <c r="F89" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G88" s="16" t="inlineStr">
+      <c r="G89" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الغطاء السحابي خلال فصل الشتاء (%)</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="17" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="18" t="inlineStr">
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="17" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
         <is>
           <t>Cld_SpMean</t>
         </is>
       </c>
-      <c r="C89" s="19" t="inlineStr">
+      <c r="C90" s="19" t="inlineStr">
         <is>
           <t>Cld_Spring_Mean</t>
         </is>
       </c>
-      <c r="D89" s="20" t="inlineStr">
+      <c r="D90" s="20" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E89" s="21" t="inlineStr">
+      <c r="E90" s="21" t="inlineStr">
         <is>
           <t>متوسط نسبة تغطية السحب لفصل الربيع الأرصادي (MAM).</t>
         </is>
       </c>
-      <c r="F89" s="22" t="inlineStr">
+      <c r="F90" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G89" s="23" t="inlineStr">
+      <c r="G90" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الغطاء السحابي خلال فصل الربيع (%)</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="10" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="11" t="inlineStr">
+    <row r="91" ht="24" customHeight="1">
+      <c r="A91" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
         <is>
           <t>Cld_SuMean</t>
         </is>
       </c>
-      <c r="C90" s="12" t="inlineStr">
+      <c r="C91" s="12" t="inlineStr">
         <is>
           <t>Cld_Summer_Mean</t>
         </is>
       </c>
-      <c r="D90" s="13" t="inlineStr">
+      <c r="D91" s="13" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E90" s="14" t="inlineStr">
+      <c r="E91" s="14" t="inlineStr">
         <is>
           <t>متوسط نسبة تغطية السحب لفصل الصيف الأرصادي (JJA).</t>
         </is>
       </c>
-      <c r="F90" s="15" t="inlineStr">
+      <c r="F91" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G90" s="16" t="inlineStr">
+      <c r="G91" s="16" t="inlineStr">
         <is>
           <t>خريطة متوسط الغطاء السحابي خلال فصل الصيف (%)</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="24" customHeight="1">
-      <c r="A91" s="17" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="18" t="inlineStr">
+    <row r="92" ht="24" customHeight="1">
+      <c r="A92" s="17" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
         <is>
           <t>Cld_AuMean</t>
         </is>
       </c>
-      <c r="C91" s="19" t="inlineStr">
+      <c r="C92" s="19" t="inlineStr">
         <is>
           <t>Cld_Autumn_Mean</t>
         </is>
       </c>
-      <c r="D91" s="20" t="inlineStr">
+      <c r="D92" s="20" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E91" s="21" t="inlineStr">
+      <c r="E92" s="21" t="inlineStr">
         <is>
           <t>متوسط نسبة تغطية السحب لفصل الخريف الأرصادي (SON).</t>
         </is>
       </c>
-      <c r="F91" s="22" t="inlineStr">
+      <c r="F92" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G91" s="23" t="inlineStr">
+      <c r="G92" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط الغطاء السحابي خلال فصل الخريف (%)</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="24" customHeight="1">
-      <c r="A92" s="10" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="11" t="inlineStr">
+    <row r="93" ht="24" customHeight="1">
+      <c r="A93" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
         <is>
           <t>Cld_AnRng</t>
         </is>
       </c>
-      <c r="C92" s="12" t="inlineStr">
+      <c r="C93" s="12" t="inlineStr">
         <is>
           <t>Cld_Annual_Range</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="D93" s="13" t="inlineStr">
         <is>
           <t>10_Cloud_Cover (الغطاء السحابي)</t>
         </is>
       </c>
-      <c r="E92" s="14" t="inlineStr">
+      <c r="E93" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي لتغطية السحب (الفارق بين أكثر شهور السنة غيوماً وأكثرها صفاءً).</t>
         </is>
       </c>
-      <c r="F92" s="15" t="inlineStr">
+      <c r="F93" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G92" s="16" t="inlineStr">
+      <c r="G93" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي لنسبة الغطاء السحابي (%)</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="24" customHeight="1">
-      <c r="A93" s="17" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="18" t="inlineStr">
+    <row r="94" ht="24" customHeight="1">
+      <c r="A94" s="17" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
         <is>
           <t>WC_WinMean</t>
         </is>
       </c>
-      <c r="C93" s="19" t="inlineStr">
+      <c r="C94" s="19" t="inlineStr">
         <is>
           <t>WC_Winter_Mean</t>
         </is>
       </c>
-      <c r="D93" s="20" t="inlineStr">
+      <c r="D94" s="20" t="inlineStr">
         <is>
           <t>12_Wind_Chill (مبرد الرياح)</t>
         </is>
       </c>
-      <c r="E93" s="21" t="inlineStr">
+      <c r="E94" s="21" t="inlineStr">
         <is>
           <t>متوسط درجة البرودة الريحية لفصل الشتاء المحسوبة بمعادلة NWS لخفض الحرارة بفعل سرعة الرياح.</t>
         </is>
       </c>
-      <c r="F93" s="22" t="inlineStr">
+      <c r="F94" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G93" s="23" t="inlineStr">
+      <c r="G94" s="23" t="inlineStr">
         <is>
           <t>خريطة متوسط مبرد الرياح خلال فصل الشتاء (°C)</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="24" customHeight="1">
-      <c r="A94" s="10" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" s="11" t="inlineStr">
+    <row r="95" ht="24" customHeight="1">
+      <c r="A95" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>WC_AnnMean</t>
         </is>
       </c>
-      <c r="C94" s="12" t="inlineStr">
+      <c r="C95" s="12" t="inlineStr">
         <is>
           <t>WC_Annual_Mean</t>
         </is>
       </c>
-      <c r="D94" s="13" t="inlineStr">
+      <c r="D95" s="13" t="inlineStr">
         <is>
           <t>12_Wind_Chill (مبرد الرياح)</t>
         </is>
       </c>
-      <c r="E94" s="14" t="inlineStr">
+      <c r="E95" s="14" t="inlineStr">
         <is>
           <t>المتوسط الحسابي السنوي لتأثير البرودة الريحية على حرارة الهواء المحسوسة.</t>
         </is>
       </c>
-      <c r="F94" s="15" t="inlineStr">
+      <c r="F95" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G94" s="16" t="inlineStr">
+      <c r="G95" s="16" t="inlineStr">
         <is>
           <t>خريطة المتوسط السنوي لمبرد الرياح (°C)</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="24" customHeight="1">
-      <c r="A95" s="17" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="18" t="inlineStr">
+    <row r="96" ht="24" customHeight="1">
+      <c r="A96" s="17" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
         <is>
           <t>DM_AridAnn</t>
         </is>
       </c>
-      <c r="C95" s="19" t="inlineStr">
+      <c r="C96" s="19" t="inlineStr">
         <is>
           <t>DM_Aridity_Annual</t>
         </is>
       </c>
-      <c r="D95" s="20" t="inlineStr">
+      <c r="D96" s="20" t="inlineStr">
         <is>
           <t>13_De_Martonne_Aridity (دليل دي مارتون)</t>
         </is>
       </c>
-      <c r="E95" s="21" t="inlineStr">
+      <c r="E96" s="21" t="inlineStr">
         <is>
           <t>دليل القحولة والجفاف السنوي لدي مارتون I = P / (T + 10) لتصنيف الأقاليم من القاحل فائق الجفاف إلى الرطب.</t>
         </is>
       </c>
-      <c r="F95" s="22" t="inlineStr">
+      <c r="F96" s="22" t="inlineStr">
         <is>
           <t>مؤشر (Index)</t>
         </is>
       </c>
-      <c r="G95" s="23" t="inlineStr">
+      <c r="G96" s="23" t="inlineStr">
         <is>
           <t>خريطة دليل دي مارتون السنوي للقحولة والجفاف</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="24" customHeight="1">
-      <c r="A96" s="10" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="11" t="inlineStr">
+    <row r="97" ht="24" customHeight="1">
+      <c r="A97" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="11" t="inlineStr">
         <is>
           <t>ET_AnnTot</t>
         </is>
       </c>
-      <c r="C96" s="12" t="inlineStr">
+      <c r="C97" s="12" t="inlineStr">
         <is>
           <t>ET_Annual_Total</t>
         </is>
       </c>
-      <c r="D96" s="13" t="inlineStr">
+      <c r="D97" s="13" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E96" s="14" t="inlineStr">
+      <c r="E97" s="14" t="inlineStr">
         <is>
           <t>المجموع التراكمي السنوي للبخر والنتح المرجعي الكامن المحسوب بمعادلة Hargreaves-Samani (FAO-56).</t>
         </is>
       </c>
-      <c r="F96" s="15" t="inlineStr">
+      <c r="F97" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G96" s="16" t="inlineStr">
+      <c r="G97" s="16" t="inlineStr">
         <is>
           <t>خريطة المجموع السنوي للبخر والنتح (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="24" customHeight="1">
-      <c r="A97" s="17" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" s="18" t="inlineStr">
+    <row r="98" ht="24" customHeight="1">
+      <c r="A98" s="17" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
         <is>
           <t>ET_AnnMean</t>
         </is>
       </c>
-      <c r="C97" s="19" t="inlineStr">
+      <c r="C98" s="19" t="inlineStr">
         <is>
           <t>ET_Annual_Mean</t>
         </is>
       </c>
-      <c r="D97" s="20" t="inlineStr">
+      <c r="D98" s="20" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E97" s="21" t="inlineStr">
+      <c r="E98" s="21" t="inlineStr">
         <is>
           <t>المعدل الشهري للبخر والنتح المرجعي (المجموع التراكمي السنوي مقسوماً على 12 شهراً).</t>
         </is>
       </c>
-      <c r="F97" s="22" t="inlineStr">
+      <c r="F98" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G97" s="23" t="inlineStr">
+      <c r="G98" s="23" t="inlineStr">
         <is>
           <t>خريطة المعدل الشهري للبخر والنتح (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="24" customHeight="1">
-      <c r="A98" s="10" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="11" t="inlineStr">
+    <row r="99" ht="24" customHeight="1">
+      <c r="A99" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
         <is>
           <t>ET_AnnRng</t>
         </is>
       </c>
-      <c r="C98" s="12" t="inlineStr">
+      <c r="C99" s="12" t="inlineStr">
         <is>
           <t>ET_Annual_Range</t>
         </is>
       </c>
-      <c r="D98" s="13" t="inlineStr">
+      <c r="D99" s="13" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E98" s="14" t="inlineStr">
+      <c r="E99" s="14" t="inlineStr">
         <is>
           <t>المدى السنوي للبخر والنتح (الفارق بين أعلى شهور السنة فقداً للماء بالبخر والنتح وأدناها).</t>
         </is>
       </c>
-      <c r="F98" s="15" t="inlineStr">
+      <c r="F99" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G98" s="16" t="inlineStr">
+      <c r="G99" s="16" t="inlineStr">
         <is>
           <t>خريطة المدى السنوي للبخر والنتح (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="24" customHeight="1">
-      <c r="A99" s="17" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="18" t="inlineStr">
+    <row r="100" ht="24" customHeight="1">
+      <c r="A100" s="17" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
         <is>
           <t>ET_SeaRng</t>
         </is>
       </c>
-      <c r="C99" s="19" t="inlineStr">
+      <c r="C100" s="19" t="inlineStr">
         <is>
           <t>ET_Seasonal_Range</t>
         </is>
       </c>
-      <c r="D99" s="20" t="inlineStr">
+      <c r="D100" s="20" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E99" s="21" t="inlineStr">
+      <c r="E100" s="21" t="inlineStr">
         <is>
           <t>المدى الفصلي للبخر والنتح (الفارق بين مجموع أعلى فصول السنة في البخر والنتح ومجموع أقلها).</t>
         </is>
       </c>
-      <c r="F99" s="22" t="inlineStr">
+      <c r="F100" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G99" s="23" t="inlineStr">
+      <c r="G100" s="23" t="inlineStr">
         <is>
           <t>خريطة المدى الفصلي للبخر والنتح (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="24" customHeight="1">
-      <c r="A100" s="10" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" s="11" t="inlineStr">
+    <row r="101" ht="24" customHeight="1">
+      <c r="A101" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
         <is>
           <t>ET_WinTot</t>
         </is>
       </c>
-      <c r="C100" s="12" t="inlineStr">
+      <c r="C101" s="12" t="inlineStr">
         <is>
           <t>ET_Winter_Total</t>
         </is>
       </c>
-      <c r="D100" s="13" t="inlineStr">
+      <c r="D101" s="13" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E100" s="14" t="inlineStr">
+      <c r="E101" s="14" t="inlineStr">
         <is>
           <t>مجموع البخر والنتح لفصل الشتاء الأرصادي (شهور ديسمبر، يناير، فبراير - DJF).</t>
         </is>
       </c>
-      <c r="F100" s="15" t="inlineStr">
+      <c r="F101" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G100" s="16" t="inlineStr">
+      <c r="G101" s="16" t="inlineStr">
         <is>
           <t>خريطة مجموع البخر والنتح خلال فصل الشتاء (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="24" customHeight="1">
-      <c r="A101" s="17" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" s="18" t="inlineStr">
+    <row r="102" ht="24" customHeight="1">
+      <c r="A102" s="17" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
         <is>
           <t>ET_SprTot</t>
         </is>
       </c>
-      <c r="C101" s="19" t="inlineStr">
+      <c r="C102" s="19" t="inlineStr">
         <is>
           <t>ET_Spring_Total</t>
         </is>
       </c>
-      <c r="D101" s="20" t="inlineStr">
+      <c r="D102" s="20" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E101" s="21" t="inlineStr">
+      <c r="E102" s="21" t="inlineStr">
         <is>
           <t>مجموع البخر والنتح لفصل الربيع الأرصادي (شهور مارس، أبريل، مايو - MAM).</t>
         </is>
       </c>
-      <c r="F101" s="22" t="inlineStr">
+      <c r="F102" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G101" s="23" t="inlineStr">
+      <c r="G102" s="23" t="inlineStr">
         <is>
           <t>خريطة مجموع البخر والنتح خلال فصل الربيع (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="24" customHeight="1">
-      <c r="A102" s="10" t="n">
-        <v>101</v>
-      </c>
-      <c r="B102" s="11" t="inlineStr">
+    <row r="103" ht="24" customHeight="1">
+      <c r="A103" s="10" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
         <is>
           <t>ET_SumTot</t>
         </is>
       </c>
-      <c r="C102" s="12" t="inlineStr">
+      <c r="C103" s="12" t="inlineStr">
         <is>
           <t>ET_Summer_Total</t>
         </is>
       </c>
-      <c r="D102" s="13" t="inlineStr">
+      <c r="D103" s="13" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E102" s="14" t="inlineStr">
+      <c r="E103" s="14" t="inlineStr">
         <is>
           <t>مجموع البخر والنتح لفصل الصيف الأرصادي (شهور يونيو، يوليو، أغسطس - JJA).</t>
         </is>
       </c>
-      <c r="F102" s="15" t="inlineStr">
+      <c r="F103" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G102" s="16" t="inlineStr">
+      <c r="G103" s="16" t="inlineStr">
         <is>
           <t>خريطة مجموع البخر والنتح خلال فصل الصيف (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="24" customHeight="1">
-      <c r="A103" s="17" t="n">
-        <v>102</v>
-      </c>
-      <c r="B103" s="18" t="inlineStr">
+    <row r="104" ht="24" customHeight="1">
+      <c r="A104" s="17" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
         <is>
           <t>ET_AutTot</t>
         </is>
       </c>
-      <c r="C103" s="19" t="inlineStr">
+      <c r="C104" s="19" t="inlineStr">
         <is>
           <t>ET_Autumn_Total</t>
         </is>
       </c>
-      <c r="D103" s="20" t="inlineStr">
+      <c r="D104" s="20" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E103" s="21" t="inlineStr">
+      <c r="E104" s="21" t="inlineStr">
         <is>
           <t>مجموع البخر والنتح لفصل الخريف الأرصادي (شهور سبتمبر، أكتوبر، نوفمبر - SON).</t>
         </is>
       </c>
-      <c r="F103" s="22" t="inlineStr">
+      <c r="F104" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G103" s="23" t="inlineStr">
+      <c r="G104" s="23" t="inlineStr">
         <is>
           <t>خريطة مجموع البخر والنتح خلال فصل الخريف (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="24" customHeight="1">
-      <c r="A104" s="10" t="n">
-        <v>103</v>
-      </c>
-      <c r="B104" s="11" t="inlineStr">
+    <row r="105" ht="24" customHeight="1">
+      <c r="A105" s="10" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
         <is>
           <t>PET_HarAnn</t>
         </is>
       </c>
-      <c r="C104" s="12" t="inlineStr">
+      <c r="C105" s="12" t="inlineStr">
         <is>
           <t>PET_Hargreaves_Annual</t>
         </is>
       </c>
-      <c r="D104" s="13" t="inlineStr">
+      <c r="D105" s="13" t="inlineStr">
         <is>
           <t>14_Evapotranspiration (البخر والنتح)</t>
         </is>
       </c>
-      <c r="E104" s="14" t="inlineStr">
+      <c r="E105" s="14" t="inlineStr">
         <is>
           <t>التبخر-نتح الكامن السنوي بهارجريفز (حقل رديف مطابق تماماً لـ ET_Annual_Total للتوافقية العكسية).</t>
         </is>
       </c>
-      <c r="F104" s="15" t="inlineStr">
+      <c r="F105" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G104" s="16" t="inlineStr">
+      <c r="G105" s="16" t="inlineStr">
         <is>
           <t>خريطة التبخر والنتح الكامن السنوي بهارجريفز (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="24" customHeight="1">
-      <c r="A105" s="17" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" s="18" t="inlineStr">
+    <row r="106" ht="24" customHeight="1">
+      <c r="A106" s="17" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
         <is>
           <t>UNEP_Arid</t>
         </is>
       </c>
-      <c r="C105" s="19" t="inlineStr">
+      <c r="C106" s="19" t="inlineStr">
         <is>
           <t>UNEP_Aridity_Annual</t>
         </is>
       </c>
-      <c r="D105" s="20" t="inlineStr">
+      <c r="D106" s="20" t="inlineStr">
         <is>
           <t>15_UNEP_Aridity (مؤشر UNEP)</t>
         </is>
       </c>
-      <c r="E105" s="21" t="inlineStr">
+      <c r="E106" s="21" t="inlineStr">
         <is>
           <t>مؤشر القحولة العالمي لبرنامج الأمم المتحدة للبيئة AI = P / ET_ann لتحديد المناطق القاحلة وشبه القاحلة.</t>
         </is>
       </c>
-      <c r="F105" s="22" t="inlineStr">
+      <c r="F106" s="22" t="inlineStr">
         <is>
           <t>نسبة (Ratio)</t>
         </is>
       </c>
-      <c r="G105" s="23" t="inlineStr">
+      <c r="G106" s="23" t="inlineStr">
         <is>
           <t>خريطة مؤشر القحولة العالمي لبرنامج الأمم المتحدة للبيئة</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="24" customHeight="1">
-      <c r="A106" s="10" t="n">
-        <v>105</v>
-      </c>
-      <c r="B106" s="11" t="inlineStr">
+    <row r="107" ht="24" customHeight="1">
+      <c r="A107" s="10" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
         <is>
           <t>WatDefAnn</t>
         </is>
       </c>
-      <c r="C106" s="12" t="inlineStr">
+      <c r="C107" s="12" t="inlineStr">
         <is>
           <t>Water_Deficit_Annual</t>
         </is>
       </c>
-      <c r="D106" s="13" t="inlineStr">
+      <c r="D107" s="13" t="inlineStr">
         <is>
           <t>16_Water_Deficit (العجز المائي)</t>
         </is>
       </c>
-      <c r="E106" s="14" t="inlineStr">
+      <c r="E107" s="14" t="inlineStr">
         <is>
           <t>الموازنة المائية المناخية السنوية الصافية WD = P - ET_ann (القيم السالبة تعبر عن عجز مائي والموجبة فائض مائي).</t>
         </is>
       </c>
-      <c r="F106" s="15" t="inlineStr">
+      <c r="F107" s="15" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G106" s="16" t="inlineStr">
+      <c r="G107" s="16" t="inlineStr">
         <is>
           <t>خريطة الموازنة والعجز المائي المناخي السنوي (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="24" customHeight="1">
-      <c r="A107" s="17" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" s="18" t="inlineStr">
+    <row r="108" ht="24" customHeight="1">
+      <c r="A108" s="17" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
         <is>
           <t>Dry_Months</t>
         </is>
       </c>
-      <c r="C107" s="19" t="inlineStr">
+      <c r="C108" s="19" t="inlineStr">
         <is>
           <t>Dry_Months_Count</t>
         </is>
       </c>
-      <c r="D107" s="20" t="inlineStr">
+      <c r="D108" s="20" t="inlineStr">
         <is>
           <t>17_Dry_Months (الأشهر الجافة)</t>
         </is>
       </c>
-      <c r="E107" s="21" t="inlineStr">
+      <c r="E108" s="21" t="inlineStr">
         <is>
           <t>عدد أشهر السنة الجافة بيولوجياً ومناخياً وفق معيار والتر-ليث البيومناخي الشهير (P &lt; 2T).</t>
         </is>
       </c>
-      <c r="F107" s="22" t="inlineStr">
+      <c r="F108" s="22" t="inlineStr">
         <is>
           <t>شهر (0-12)</t>
         </is>
       </c>
-      <c r="G107" s="23" t="inlineStr">
+      <c r="G108" s="23" t="inlineStr">
         <is>
           <t>خريطة عدد الأشهر الجافة بيولوجياً في السنة</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="24" customHeight="1">
-      <c r="A108" s="10" t="n">
-        <v>107</v>
-      </c>
-      <c r="B108" s="11" t="inlineStr">
+    <row r="109" ht="24" customHeight="1">
+      <c r="A109" s="10" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
         <is>
           <t>T_TrendDec</t>
         </is>
       </c>
-      <c r="C108" s="12" t="inlineStr">
+      <c r="C109" s="12" t="inlineStr">
         <is>
           <t>T_Trend_Decade</t>
         </is>
       </c>
-      <c r="D108" s="13" t="inlineStr">
+      <c r="D109" s="13" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E108" s="14" t="inlineStr">
+      <c r="E109" s="14" t="inlineStr">
         <is>
           <t>معدل تغير واتجاه درجة الحرارة لكل عقد زمني (10 سنوات) باستخدام انحدار المربعات الصغرى الخطي.</t>
         </is>
       </c>
-      <c r="F108" s="15" t="inlineStr">
+      <c r="F109" s="15" t="inlineStr">
         <is>
           <t>°C/decade</t>
         </is>
       </c>
-      <c r="G108" s="16" t="inlineStr">
+      <c r="G109" s="16" t="inlineStr">
         <is>
           <t>خريطة اتجاه تغير درجة الحرارة في العقد الزمني (°C/decade)</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="24" customHeight="1">
-      <c r="A109" s="17" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" s="18" t="inlineStr">
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="17" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
         <is>
           <t>R_TrendDec</t>
         </is>
       </c>
-      <c r="C109" s="19" t="inlineStr">
+      <c r="C110" s="19" t="inlineStr">
         <is>
           <t>R_Trend_Decade</t>
         </is>
       </c>
-      <c r="D109" s="20" t="inlineStr">
+      <c r="D110" s="20" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E109" s="21" t="inlineStr">
+      <c r="E110" s="21" t="inlineStr">
         <is>
           <t>معدل تغير واتجاه تساقط الأمطار لكل عقد زمني (10 سنوات) باستخدام انحدار المربعات الصغرى الخطي.</t>
         </is>
       </c>
-      <c r="F109" s="22" t="inlineStr">
+      <c r="F110" s="22" t="inlineStr">
         <is>
           <t>mm/decade</t>
         </is>
       </c>
-      <c r="G109" s="23" t="inlineStr">
+      <c r="G110" s="23" t="inlineStr">
         <is>
           <t>خريطة اتجاه تغير تساقط الأمطار في العقد الزمني (mm/decade)</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="24" customHeight="1">
-      <c r="A110" s="10" t="n">
-        <v>109</v>
-      </c>
-      <c r="B110" s="11" t="inlineStr">
+    <row r="111" ht="24" customHeight="1">
+      <c r="A111" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
         <is>
           <t>T_AnomAnn</t>
         </is>
       </c>
-      <c r="C110" s="12" t="inlineStr">
+      <c r="C111" s="12" t="inlineStr">
         <is>
           <t>T_Anom_Annual</t>
         </is>
       </c>
-      <c r="D110" s="13" t="inlineStr">
+      <c r="D111" s="13" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E110" s="14" t="inlineStr">
+      <c r="E111" s="14" t="inlineStr">
         <is>
           <t>الشذوذ الحراري السنوي لدرجة الحرارة مقارنة بخط الأساس المناخي العالمي 1991–2020.</t>
         </is>
       </c>
-      <c r="F110" s="15" t="inlineStr">
+      <c r="F111" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G110" s="16" t="inlineStr">
+      <c r="G111" s="16" t="inlineStr">
         <is>
           <t>خريطة الشذوذ الحراري السنوي مقارنة بخط أساس 1991–2020 (°C)</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="24" customHeight="1">
-      <c r="A111" s="17" t="n">
-        <v>110</v>
-      </c>
-      <c r="B111" s="18" t="inlineStr">
+    <row r="112" ht="24" customHeight="1">
+      <c r="A112" s="17" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="18" t="inlineStr">
         <is>
           <t>T_AnomWin</t>
         </is>
       </c>
-      <c r="C111" s="19" t="inlineStr">
+      <c r="C112" s="19" t="inlineStr">
         <is>
           <t>T_Anom_Winter</t>
         </is>
       </c>
-      <c r="D111" s="20" t="inlineStr">
+      <c r="D112" s="20" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E111" s="21" t="inlineStr">
+      <c r="E112" s="21" t="inlineStr">
         <is>
           <t>الشذوذ الحراري لفصل الشتاء مقارنة بمتوسط شهور الشتاء لخط الأساس المناخي 1991–2020.</t>
         </is>
       </c>
-      <c r="F111" s="22" t="inlineStr">
+      <c r="F112" s="22" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G111" s="23" t="inlineStr">
+      <c r="G112" s="23" t="inlineStr">
         <is>
           <t>خريطة الشذوذ الحراري لفصل الشتاء مقارنة بخط أساس 1991–2020 (°C)</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="24" customHeight="1">
-      <c r="A112" s="10" t="n">
-        <v>111</v>
-      </c>
-      <c r="B112" s="11" t="inlineStr">
+    <row r="113" ht="24" customHeight="1">
+      <c r="A113" s="10" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
         <is>
           <t>T_AnomSum</t>
         </is>
       </c>
-      <c r="C112" s="12" t="inlineStr">
+      <c r="C113" s="12" t="inlineStr">
         <is>
           <t>T_Anom_Summer</t>
         </is>
       </c>
-      <c r="D112" s="13" t="inlineStr">
+      <c r="D113" s="13" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E112" s="14" t="inlineStr">
+      <c r="E113" s="14" t="inlineStr">
         <is>
           <t>الشذوذ الحراري لفصل الصيف مقارنة بمتوسط شهور الصيف لخط الأساس المناخي 1991–2020.</t>
         </is>
       </c>
-      <c r="F112" s="15" t="inlineStr">
+      <c r="F113" s="15" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G112" s="16" t="inlineStr">
+      <c r="G113" s="16" t="inlineStr">
         <is>
           <t>خريطة الشذوذ الحراري لفصل الصيف مقارنة بخط أساس 1991–2020 (°C)</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="24" customHeight="1">
-      <c r="A113" s="17" t="n">
-        <v>112</v>
-      </c>
-      <c r="B113" s="18" t="inlineStr">
+    <row r="114" ht="24" customHeight="1">
+      <c r="A114" s="17" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="18" t="inlineStr">
         <is>
           <t>R_AnomAnn</t>
         </is>
       </c>
-      <c r="C113" s="19" t="inlineStr">
+      <c r="C114" s="19" t="inlineStr">
         <is>
           <t>R_Anom_Annual</t>
         </is>
       </c>
-      <c r="D113" s="20" t="inlineStr">
+      <c r="D114" s="20" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E113" s="21" t="inlineStr">
+      <c r="E114" s="21" t="inlineStr">
         <is>
           <t>شذوذ الأمطار السنوي المطلق مقارنة بمتوسط الأمطار لخط الأساس المناخي 1991–2020.</t>
         </is>
       </c>
-      <c r="F113" s="22" t="inlineStr">
+      <c r="F114" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G113" s="23" t="inlineStr">
+      <c r="G114" s="23" t="inlineStr">
         <is>
           <t>خريطة شذوذ تساقط الأمطار السنوي مقارنة بخط أساس 1991–2020 (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="24" customHeight="1">
-      <c r="A114" s="10" t="n">
-        <v>113</v>
-      </c>
-      <c r="B114" s="11" t="inlineStr">
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="10" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
         <is>
           <t>R_AnomPct</t>
         </is>
       </c>
-      <c r="C114" s="12" t="inlineStr">
+      <c r="C115" s="12" t="inlineStr">
         <is>
           <t>R_Anom_Annual_Pct</t>
         </is>
       </c>
-      <c r="D114" s="13" t="inlineStr">
+      <c r="D115" s="13" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E114" s="14" t="inlineStr">
+      <c r="E115" s="14" t="inlineStr">
         <is>
           <t>شذوذ الأمطار السنوي كنسبة مئوية من خط الأساس المناخي 1991–2020 (فرق نسبي مئوي).</t>
         </is>
       </c>
-      <c r="F114" s="15" t="inlineStr">
+      <c r="F115" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G114" s="16" t="inlineStr">
+      <c r="G115" s="16" t="inlineStr">
         <is>
           <t>خريطة الشذوذ النسبي المئوي للأمطار مقارنة بخط أساس 1991–2020 (%)</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="24" customHeight="1">
-      <c r="A115" s="17" t="n">
-        <v>114</v>
-      </c>
-      <c r="B115" s="18" t="inlineStr">
+    <row r="116" ht="24" customHeight="1">
+      <c r="A116" s="17" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="18" t="inlineStr">
         <is>
           <t>R_AnomWin</t>
         </is>
       </c>
-      <c r="C115" s="19" t="inlineStr">
+      <c r="C116" s="19" t="inlineStr">
         <is>
           <t>R_Anom_Winter</t>
         </is>
       </c>
-      <c r="D115" s="20" t="inlineStr">
+      <c r="D116" s="20" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E115" s="21" t="inlineStr">
+      <c r="E116" s="21" t="inlineStr">
         <is>
           <t>شذوذ أمطار فصل الشتاء المطلق مقارنة بأمطار شتاء خط الأساس المناخي 1991–2020.</t>
         </is>
       </c>
-      <c r="F115" s="22" t="inlineStr">
+      <c r="F116" s="22" t="inlineStr">
         <is>
           <t>ملم (mm)</t>
         </is>
       </c>
-      <c r="G115" s="23" t="inlineStr">
+      <c r="G116" s="23" t="inlineStr">
         <is>
           <t>خريطة شذوذ أمطار الشتاء مقارنة بخط أساس 1991–2020 (ملم)</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="24" customHeight="1">
-      <c r="A116" s="10" t="n">
-        <v>115</v>
-      </c>
-      <c r="B116" s="11" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="10" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
         <is>
           <t>R_AnomWPct</t>
         </is>
       </c>
-      <c r="C116" s="12" t="inlineStr">
+      <c r="C117" s="12" t="inlineStr">
         <is>
           <t>R_Anom_Winter_Pct</t>
         </is>
       </c>
-      <c r="D116" s="13" t="inlineStr">
+      <c r="D117" s="13" t="inlineStr">
         <is>
           <t>18_Trends_And_Anomalies (الاتجاهات والشذوذ)</t>
         </is>
       </c>
-      <c r="E116" s="14" t="inlineStr">
+      <c r="E117" s="14" t="inlineStr">
         <is>
           <t>شذوذ أمطار فصل الشتاء كنسبة مئوية مقارنة بأمطار شتاء خط الأساس المناخي 1991–2020.</t>
         </is>
       </c>
-      <c r="F116" s="15" t="inlineStr">
+      <c r="F117" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G116" s="16" t="inlineStr">
+      <c r="G117" s="16" t="inlineStr">
         <is>
           <t>خريطة الشذوذ النسبي المئوي لأمطار الشتاء مقارنة بخط أساس 1991–2020 (%)</t>
         </is>

</xml_diff>